<commit_message>
feat(owas): time picker rotella + rimozione postazione + fix numFmt template
- DurationPicker: nuovo componente scroll-wheel (ore + minuti a step di 5)
  sostituisce l'input testo libero; durata diventa number|null (minuti)
- MisuraOwasModal: rimosso campo postazione (hook, stato, modal, buildDati)
  integrato DurationPicker; isValid ora dipende da durata invece di postazioneId
- exportSchemas (OWAS): cella D (durata hh:mm:ss) scritta per ultima, dopo E-I,
  per evitare ereditarietà xfId che sovrascriveva numFmt sulle celle numeriche
- owas.xlsx template: rigenerato con script fix-owas-template.py
- tools/: aggiunti inspect-owas-template.py e fix-owas-template.py (diagnostica)
- .gitignore: aggiunto *.bak

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/templates/owas.xlsx
+++ b/public/templates/owas.xlsx
@@ -18,7 +18,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="[hh]:mm:ss"/>
+  </numFmts>
   <fonts count="4">
     <font>
       <name val="Calibri"/>
@@ -60,7 +62,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="9">
     <border>
       <left/>
       <right/>
@@ -82,11 +84,88 @@
         <color rgb="00000000"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="00000000"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="00000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00000000"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="00000000"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="00000000"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color rgb="00000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -115,6 +194,15 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -550,10 +638,10 @@
           <t>CODICE OWAS</t>
         </is>
       </c>
-      <c r="F3" s="6" t="n"/>
-      <c r="G3" s="6" t="n"/>
-      <c r="H3" s="6" t="n"/>
-      <c r="I3" s="6" t="n"/>
+      <c r="F3" s="11" t="n"/>
+      <c r="G3" s="11" t="n"/>
+      <c r="H3" s="11" t="n"/>
+      <c r="I3" s="12" t="n"/>
       <c r="J3" s="5" t="inlineStr">
         <is>
           <t>NOTE</t>
@@ -561,10 +649,10 @@
       </c>
     </row>
     <row r="4" ht="18" customHeight="1">
-      <c r="A4" s="6" t="n"/>
-      <c r="B4" s="6" t="n"/>
-      <c r="C4" s="6" t="n"/>
-      <c r="D4" s="6" t="n"/>
+      <c r="A4" s="13" t="n"/>
+      <c r="B4" s="13" t="n"/>
+      <c r="C4" s="13" t="n"/>
+      <c r="D4" s="13" t="n"/>
       <c r="E4" s="5" t="inlineStr">
         <is>
           <t>SCHIENA</t>
@@ -590,7 +678,7 @@
           <t>CLASSE</t>
         </is>
       </c>
-      <c r="J4" s="6" t="n"/>
+      <c r="J4" s="13" t="n"/>
     </row>
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="7" t="n">
@@ -598,12 +686,12 @@
       </c>
       <c r="B5" s="8" t="n"/>
       <c r="C5" s="8" t="n"/>
-      <c r="D5" s="8" t="n"/>
-      <c r="E5" s="8" t="n"/>
-      <c r="F5" s="8" t="n"/>
-      <c r="G5" s="8" t="n"/>
-      <c r="H5" s="8" t="n"/>
-      <c r="I5" s="8" t="n"/>
+      <c r="D5" s="14" t="n"/>
+      <c r="E5" s="15" t="n"/>
+      <c r="F5" s="15" t="n"/>
+      <c r="G5" s="15" t="n"/>
+      <c r="H5" s="15" t="n"/>
+      <c r="I5" s="15" t="n"/>
       <c r="J5" s="8" t="n"/>
     </row>
     <row r="6" ht="30" customHeight="1">
@@ -612,12 +700,12 @@
       </c>
       <c r="B6" s="8" t="n"/>
       <c r="C6" s="8" t="n"/>
-      <c r="D6" s="8" t="n"/>
-      <c r="E6" s="8" t="n"/>
-      <c r="F6" s="8" t="n"/>
-      <c r="G6" s="8" t="n"/>
-      <c r="H6" s="8" t="n"/>
-      <c r="I6" s="8" t="n"/>
+      <c r="D6" s="14" t="n"/>
+      <c r="E6" s="15" t="n"/>
+      <c r="F6" s="15" t="n"/>
+      <c r="G6" s="15" t="n"/>
+      <c r="H6" s="15" t="n"/>
+      <c r="I6" s="15" t="n"/>
       <c r="J6" s="8" t="n"/>
     </row>
     <row r="7" ht="30" customHeight="1">
@@ -626,12 +714,12 @@
       </c>
       <c r="B7" s="8" t="n"/>
       <c r="C7" s="8" t="n"/>
-      <c r="D7" s="8" t="n"/>
-      <c r="E7" s="8" t="n"/>
-      <c r="F7" s="8" t="n"/>
-      <c r="G7" s="8" t="n"/>
-      <c r="H7" s="8" t="n"/>
-      <c r="I7" s="8" t="n"/>
+      <c r="D7" s="14" t="n"/>
+      <c r="E7" s="15" t="n"/>
+      <c r="F7" s="15" t="n"/>
+      <c r="G7" s="15" t="n"/>
+      <c r="H7" s="15" t="n"/>
+      <c r="I7" s="15" t="n"/>
       <c r="J7" s="8" t="n"/>
     </row>
     <row r="8" ht="30" customHeight="1">
@@ -640,12 +728,12 @@
       </c>
       <c r="B8" s="8" t="n"/>
       <c r="C8" s="8" t="n"/>
-      <c r="D8" s="8" t="n"/>
-      <c r="E8" s="8" t="n"/>
-      <c r="F8" s="8" t="n"/>
-      <c r="G8" s="8" t="n"/>
-      <c r="H8" s="8" t="n"/>
-      <c r="I8" s="8" t="n"/>
+      <c r="D8" s="14" t="n"/>
+      <c r="E8" s="15" t="n"/>
+      <c r="F8" s="15" t="n"/>
+      <c r="G8" s="15" t="n"/>
+      <c r="H8" s="15" t="n"/>
+      <c r="I8" s="15" t="n"/>
       <c r="J8" s="8" t="n"/>
     </row>
     <row r="9" ht="30" customHeight="1">
@@ -654,12 +742,12 @@
       </c>
       <c r="B9" s="8" t="n"/>
       <c r="C9" s="8" t="n"/>
-      <c r="D9" s="8" t="n"/>
-      <c r="E9" s="8" t="n"/>
-      <c r="F9" s="8" t="n"/>
-      <c r="G9" s="8" t="n"/>
-      <c r="H9" s="8" t="n"/>
-      <c r="I9" s="8" t="n"/>
+      <c r="D9" s="14" t="n"/>
+      <c r="E9" s="15" t="n"/>
+      <c r="F9" s="15" t="n"/>
+      <c r="G9" s="15" t="n"/>
+      <c r="H9" s="15" t="n"/>
+      <c r="I9" s="15" t="n"/>
       <c r="J9" s="8" t="n"/>
     </row>
     <row r="10" ht="30" customHeight="1">
@@ -668,12 +756,12 @@
       </c>
       <c r="B10" s="8" t="n"/>
       <c r="C10" s="8" t="n"/>
-      <c r="D10" s="8" t="n"/>
-      <c r="E10" s="8" t="n"/>
-      <c r="F10" s="8" t="n"/>
-      <c r="G10" s="8" t="n"/>
-      <c r="H10" s="8" t="n"/>
-      <c r="I10" s="8" t="n"/>
+      <c r="D10" s="14" t="n"/>
+      <c r="E10" s="15" t="n"/>
+      <c r="F10" s="15" t="n"/>
+      <c r="G10" s="15" t="n"/>
+      <c r="H10" s="15" t="n"/>
+      <c r="I10" s="15" t="n"/>
       <c r="J10" s="8" t="n"/>
     </row>
     <row r="11" ht="30" customHeight="1">
@@ -682,12 +770,12 @@
       </c>
       <c r="B11" s="8" t="n"/>
       <c r="C11" s="8" t="n"/>
-      <c r="D11" s="8" t="n"/>
-      <c r="E11" s="8" t="n"/>
-      <c r="F11" s="8" t="n"/>
-      <c r="G11" s="8" t="n"/>
-      <c r="H11" s="8" t="n"/>
-      <c r="I11" s="8" t="n"/>
+      <c r="D11" s="14" t="n"/>
+      <c r="E11" s="15" t="n"/>
+      <c r="F11" s="15" t="n"/>
+      <c r="G11" s="15" t="n"/>
+      <c r="H11" s="15" t="n"/>
+      <c r="I11" s="15" t="n"/>
       <c r="J11" s="8" t="n"/>
     </row>
     <row r="12" ht="30" customHeight="1">
@@ -696,12 +784,12 @@
       </c>
       <c r="B12" s="8" t="n"/>
       <c r="C12" s="8" t="n"/>
-      <c r="D12" s="8" t="n"/>
-      <c r="E12" s="8" t="n"/>
-      <c r="F12" s="8" t="n"/>
-      <c r="G12" s="8" t="n"/>
-      <c r="H12" s="8" t="n"/>
-      <c r="I12" s="8" t="n"/>
+      <c r="D12" s="14" t="n"/>
+      <c r="E12" s="15" t="n"/>
+      <c r="F12" s="15" t="n"/>
+      <c r="G12" s="15" t="n"/>
+      <c r="H12" s="15" t="n"/>
+      <c r="I12" s="15" t="n"/>
       <c r="J12" s="8" t="n"/>
     </row>
     <row r="13" ht="15" customHeight="1"/>
@@ -717,8 +805,8 @@
   <mergeCells count="10">
     <mergeCell ref="E3:I3"/>
     <mergeCell ref="C3:C4"/>
+    <mergeCell ref="A3:A4"/>
     <mergeCell ref="B3:B4"/>
-    <mergeCell ref="A3:A4"/>
     <mergeCell ref="D3:D4"/>
     <mergeCell ref="J3:J4"/>
     <mergeCell ref="A14:B14"/>

</xml_diff>